<commit_message>
Data profiling: tabela categories
</commit_message>
<xml_diff>
--- a/docs/profiling/problemas_qualidade.xlsx
+++ b/docs/profiling/problemas_qualidade.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="620" uniqueCount="311">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="649" uniqueCount="327">
   <si>
     <t xml:space="preserve">Data Profiling — Problemas de Qualidade dos Dados (MoreRhythm)</t>
   </si>
@@ -723,6 +723,24 @@
     <t xml:space="preserve">"Aparelhos Electrónicos" (Rádios) usa a grafia anterior ao Acordo Ortográfico; não é erro, mas pode ser normalizado.</t>
   </si>
   <si>
+    <t xml:space="preserve">categories</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Category</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Siglas escritas em minúsculas, de forma inconsistente com a grafia habitual</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Leitor de Cd" e "Leitor de Mp3" (em vez de "Leitor de CD" / "Leitor de MP3")</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Normalizar através de tabela de mapeamento de valores na transformação</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Problema apenas de apresentação; não afeta agrupamentos nem análises.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Resumo dos problemas encontrados</t>
   </si>
   <si>
@@ -738,9 +756,6 @@
     <t xml:space="preserve">products</t>
   </si>
   <si>
-    <t xml:space="preserve">categories</t>
-  </si>
-  <si>
     <t xml:space="preserve">suplliers</t>
   </si>
   <si>
@@ -943,6 +958,39 @@
   </si>
   <si>
     <t xml:space="preserve">Todos os produtos com família preenchida referem uma família existente. Os produtos sem família (Z001 e CORSR, com todos os atributos a NULL) são tratados na análise da products.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tabela limpa: código e Category 100% únicos, sem NULLs nem vazios, códigos consecutivos de 1 a 11. Todos os produtos com categoria preenchida referem uma categoria existente (os produtos Z001 e CORSR, sem categoria, são tratados na products).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Candidate Key + Column Statistics + SQL b)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A tabela não tem datas de criação nem de alteração: a carga incremental não pode basear-se em datas; é preciso comparar os registos (ex.: componente Slowly Changing Dimension ou Lookup sobre o código).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Estrutura da tabela</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 categoria sem produtos: "Complementos" (código 3).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As categorias da análise 9 ("Ar", "Cordas" e "Membranas") existem e têm vendas (10, 27 e 11 linhas de fatura, respetivamente).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SQL c)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Família e categoria não formam uma hierarquia: a família Acessorios tem produtos em 4 categorias (Cases, Cordas, Interface, Peças) e as categorias Cordas e Peças têm produtos de 2 famílias. No modelo dimensional devem ser duas hierarquias independentes na dimensão produto (produto → família e produto → categoria).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SQL d)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Peças" e "Pilhas" existem simultaneamente como categoria, como família/classificação ou como classification dos produtos. Convém nomear claramente os atributos na dimensão para evitar confusão nas análises.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Comparação entre tabelas</t>
   </si>
   <si>
     <t xml:space="preserve">Perfil</t>
@@ -3327,23 +3375,47 @@
         <v>230</v>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="7" t="str">
+    <row r="44" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="7" t="n">
         <f aca="false">IF(B44="","",COUNTA($B$5:B44))</f>
-        <v/>
-      </c>
-      <c r="B44" s="8"/>
-      <c r="C44" s="8"/>
-      <c r="D44" s="8"/>
-      <c r="E44" s="8"/>
-      <c r="F44" s="8"/>
-      <c r="G44" s="9"/>
-      <c r="H44" s="8"/>
-      <c r="I44" s="9"/>
-      <c r="J44" s="9"/>
-      <c r="K44" s="8"/>
-      <c r="L44" s="8"/>
-      <c r="M44" s="8"/>
+        <v>40</v>
+      </c>
+      <c r="B44" s="8" t="s">
+        <v>231</v>
+      </c>
+      <c r="C44" s="8" t="s">
+        <v>232</v>
+      </c>
+      <c r="D44" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="E44" s="8" t="s">
+        <v>233</v>
+      </c>
+      <c r="F44" s="8" t="s">
+        <v>234</v>
+      </c>
+      <c r="G44" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="H44" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="I44" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="J44" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="K44" s="8" t="s">
+        <v>235</v>
+      </c>
+      <c r="L44" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="M44" s="8" t="s">
+        <v>236</v>
+      </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="4" t="str">
@@ -5401,7 +5473,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>231</v>
+        <v>237</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -5411,7 +5483,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="10" t="s">
-        <v>232</v>
+        <v>238</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5428,10 +5500,10 @@
         <v>55</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>233</v>
+        <v>239</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>234</v>
+        <v>240</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5511,7 +5583,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="11" t="s">
-        <v>235</v>
+        <v>241</v>
       </c>
       <c r="B8" s="12" t="n">
         <f aca="false">COUNTIFS(Problemas!$B$5:$B$154,$A8,Problemas!$I$5:$I$154,"Alta")</f>
@@ -5561,7 +5633,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="11" t="s">
-        <v>236</v>
+        <v>231</v>
       </c>
       <c r="B10" s="12" t="n">
         <f aca="false">COUNTIFS(Problemas!$B$5:$B$154,$A10,Problemas!$I$5:$I$154,"Alta")</f>
@@ -5573,20 +5645,20 @@
       </c>
       <c r="D10" s="12" t="n">
         <f aca="false">COUNTIFS(Problemas!$B$5:$B$154,$A10,Problemas!$I$5:$I$154,"Baixa")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E10" s="12" t="n">
         <f aca="false">COUNTIF(Problemas!$B$5:$B$154,$A10)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F10" s="12" t="n">
         <f aca="false">SUMIF(Problemas!$B$5:$B$154,$A10,Problemas!$G$5:$G$154)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="11" t="s">
-        <v>237</v>
+        <v>242</v>
       </c>
       <c r="B11" s="12" t="n">
         <f aca="false">COUNTIFS(Problemas!$B$5:$B$154,$A11,Problemas!$I$5:$I$154,"Alta")</f>
@@ -5611,7 +5683,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="11" t="s">
-        <v>238</v>
+        <v>243</v>
       </c>
       <c r="B12" s="12" t="n">
         <f aca="false">COUNTIFS(Problemas!$B$5:$B$154,$A12,Problemas!$I$5:$I$154,"Alta")</f>
@@ -5636,7 +5708,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="11" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="B13" s="12" t="n">
         <f aca="false">COUNTIFS(Problemas!$B$5:$B$154,$A13,Problemas!$I$5:$I$154,"Alta")</f>
@@ -5661,7 +5733,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="13" t="s">
-        <v>233</v>
+        <v>239</v>
       </c>
       <c r="B14" s="14" t="n">
         <f aca="false">SUM(B5:B13)</f>
@@ -5673,15 +5745,15 @@
       </c>
       <c r="D14" s="14" t="n">
         <f aca="false">SUM(D5:D13)</f>
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E14" s="14" t="n">
         <f aca="false">SUM(E5:E13)</f>
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F14" s="14" t="n">
         <f aca="false">SUM(F5:F13)</f>
-        <v>490</v>
+        <v>492</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5689,13 +5761,13 @@
         <v>9</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>240</v>
+        <v>245</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>241</v>
+        <v>246</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>242</v>
+        <v>247</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5755,11 +5827,11 @@
       </c>
       <c r="B21" s="12" t="n">
         <f aca="false">COUNTIF(Problemas!$H$5:$H$154,$A21)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C21" s="12" t="n">
         <f aca="false">COUNTIFS(Problemas!$H$5:$H$154,$A21,Problemas!$J$5:$J$154,"Sim")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D21" s="12" t="n">
         <f aca="false">COUNTIFS(Problemas!$H$5:$H$154,$A21,Problemas!$L$5:$L$154,"Tabela de erros (SA)")</f>
@@ -5853,15 +5925,15 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="13" t="s">
-        <v>233</v>
+        <v>239</v>
       </c>
       <c r="B27" s="14" t="n">
         <f aca="false">SUM(B18:B26)</f>
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C27" s="14" t="n">
         <f aca="false">SUM(C18:C26)</f>
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D27" s="14" t="n">
         <f aca="false">SUM(D18:D26)</f>
@@ -5897,7 +5969,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>243</v>
+        <v>248</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -5907,21 +5979,21 @@
         <v>4</v>
       </c>
       <c r="B3" s="15" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="C3" s="15" t="s">
-        <v>245</v>
+        <v>250</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="16" t="s">
-        <v>246</v>
+        <v>251</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>247</v>
+        <v>252</v>
       </c>
       <c r="C4" s="17" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5929,7 +6001,7 @@
         <v>5</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="C5" s="17" t="s">
         <v>39</v>
@@ -5940,21 +6012,21 @@
         <v>6</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>250</v>
+        <v>255</v>
       </c>
       <c r="C6" s="17" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="16" t="s">
-        <v>245</v>
+        <v>250</v>
       </c>
       <c r="B7" s="17" t="s">
-        <v>252</v>
+        <v>257</v>
       </c>
       <c r="C7" s="17" t="s">
-        <v>253</v>
+        <v>258</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5962,10 +6034,10 @@
         <v>8</v>
       </c>
       <c r="B8" s="17" t="s">
-        <v>254</v>
+        <v>259</v>
       </c>
       <c r="C8" s="17" t="s">
-        <v>255</v>
+        <v>260</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5973,7 +6045,7 @@
         <v>9</v>
       </c>
       <c r="B9" s="17" t="s">
-        <v>256</v>
+        <v>261</v>
       </c>
       <c r="C9" s="17" t="s">
         <v>42</v>
@@ -5984,7 +6056,7 @@
         <v>10</v>
       </c>
       <c r="B10" s="17" t="s">
-        <v>257</v>
+        <v>262</v>
       </c>
       <c r="C10" s="17" t="s">
         <v>43</v>
@@ -5995,7 +6067,7 @@
         <v>11</v>
       </c>
       <c r="B11" s="17" t="s">
-        <v>258</v>
+        <v>263</v>
       </c>
       <c r="C11" s="17" t="s">
         <v>92</v>
@@ -6003,13 +6075,13 @@
     </row>
     <row r="12" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="16" t="s">
-        <v>259</v>
+        <v>264</v>
       </c>
       <c r="B12" s="17" t="s">
-        <v>260</v>
+        <v>265</v>
       </c>
       <c r="C12" s="17" t="s">
-        <v>261</v>
+        <v>266</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6017,7 +6089,7 @@
         <v>13</v>
       </c>
       <c r="B13" s="17" t="s">
-        <v>262</v>
+        <v>267</v>
       </c>
       <c r="C13" s="17" t="s">
         <v>24</v>
@@ -6042,7 +6114,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C42"/>
+  <dimension ref="A1:C48"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16"/>
@@ -6052,7 +6124,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>263</v>
+        <v>268</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -6062,10 +6134,10 @@
         <v>3</v>
       </c>
       <c r="B3" s="18" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
       <c r="C3" s="18" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6073,10 +6145,10 @@
         <v>15</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="C4" s="19" t="s">
-        <v>267</v>
+        <v>272</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6084,10 +6156,10 @@
         <v>15</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>268</v>
+        <v>273</v>
       </c>
       <c r="C5" s="19" t="s">
-        <v>269</v>
+        <v>274</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6095,10 +6167,10 @@
         <v>15</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>270</v>
+        <v>275</v>
       </c>
       <c r="C6" s="19" t="s">
-        <v>271</v>
+        <v>276</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6106,7 +6178,7 @@
         <v>15</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
       <c r="C7" s="19" t="s">
         <v>27</v>
@@ -6117,10 +6189,10 @@
         <v>15</v>
       </c>
       <c r="B8" s="19" t="s">
-        <v>273</v>
+        <v>278</v>
       </c>
       <c r="C8" s="19" t="s">
-        <v>274</v>
+        <v>279</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6128,7 +6200,7 @@
         <v>15</v>
       </c>
       <c r="B9" s="19" t="s">
-        <v>275</v>
+        <v>280</v>
       </c>
       <c r="C9" s="19" t="s">
         <v>141</v>
@@ -6139,10 +6211,10 @@
         <v>15</v>
       </c>
       <c r="B10" s="19" t="s">
-        <v>276</v>
+        <v>281</v>
       </c>
       <c r="C10" s="19" t="s">
-        <v>277</v>
+        <v>282</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6150,10 +6222,10 @@
         <v>129</v>
       </c>
       <c r="B11" s="19" t="s">
-        <v>278</v>
+        <v>283</v>
       </c>
       <c r="C11" s="19" t="s">
-        <v>279</v>
+        <v>284</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6161,10 +6233,10 @@
         <v>129</v>
       </c>
       <c r="B12" s="19" t="s">
-        <v>280</v>
+        <v>285</v>
       </c>
       <c r="C12" s="19" t="s">
-        <v>281</v>
+        <v>286</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6172,10 +6244,10 @@
         <v>129</v>
       </c>
       <c r="B13" s="19" t="s">
-        <v>282</v>
+        <v>287</v>
       </c>
       <c r="C13" s="19" t="s">
-        <v>283</v>
+        <v>288</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6183,10 +6255,10 @@
         <v>129</v>
       </c>
       <c r="B14" s="19" t="s">
-        <v>284</v>
+        <v>289</v>
       </c>
       <c r="C14" s="19" t="s">
-        <v>285</v>
+        <v>290</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6194,10 +6266,10 @@
         <v>129</v>
       </c>
       <c r="B15" s="19" t="s">
-        <v>286</v>
+        <v>291</v>
       </c>
       <c r="C15" s="19" t="s">
-        <v>287</v>
+        <v>292</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6205,10 +6277,10 @@
         <v>129</v>
       </c>
       <c r="B16" s="19" t="s">
-        <v>288</v>
+        <v>293</v>
       </c>
       <c r="C16" s="19" t="s">
-        <v>277</v>
+        <v>282</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6216,10 +6288,10 @@
         <v>167</v>
       </c>
       <c r="B17" s="19" t="s">
-        <v>289</v>
+        <v>294</v>
       </c>
       <c r="C17" s="19" t="s">
-        <v>290</v>
+        <v>295</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6227,7 +6299,7 @@
         <v>167</v>
       </c>
       <c r="B18" s="19" t="s">
-        <v>291</v>
+        <v>296</v>
       </c>
       <c r="C18" s="19" t="s">
         <v>141</v>
@@ -6238,7 +6310,7 @@
         <v>167</v>
       </c>
       <c r="B19" s="19" t="s">
-        <v>292</v>
+        <v>297</v>
       </c>
       <c r="C19" s="19" t="s">
         <v>141</v>
@@ -6249,10 +6321,10 @@
         <v>167</v>
       </c>
       <c r="B20" s="19" t="s">
-        <v>293</v>
+        <v>298</v>
       </c>
       <c r="C20" s="19" t="s">
-        <v>294</v>
+        <v>299</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6260,7 +6332,7 @@
         <v>167</v>
       </c>
       <c r="B21" s="19" t="s">
-        <v>295</v>
+        <v>300</v>
       </c>
       <c r="C21" s="19" t="s">
         <v>141</v>
@@ -6271,7 +6343,7 @@
         <v>167</v>
       </c>
       <c r="B22" s="19" t="s">
-        <v>296</v>
+        <v>301</v>
       </c>
       <c r="C22" s="19" t="s">
         <v>141</v>
@@ -6282,10 +6354,10 @@
         <v>167</v>
       </c>
       <c r="B23" s="19" t="s">
-        <v>297</v>
+        <v>302</v>
       </c>
       <c r="C23" s="19" t="s">
-        <v>277</v>
+        <v>282</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6293,10 +6365,10 @@
         <v>211</v>
       </c>
       <c r="B24" s="19" t="s">
-        <v>298</v>
+        <v>303</v>
       </c>
       <c r="C24" s="19" t="s">
-        <v>299</v>
+        <v>304</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6304,10 +6376,10 @@
         <v>211</v>
       </c>
       <c r="B25" s="19" t="s">
-        <v>300</v>
+        <v>305</v>
       </c>
       <c r="C25" s="19" t="s">
-        <v>301</v>
+        <v>306</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6315,10 +6387,10 @@
         <v>211</v>
       </c>
       <c r="B26" s="19" t="s">
-        <v>302</v>
+        <v>307</v>
       </c>
       <c r="C26" s="19" t="s">
-        <v>303</v>
+        <v>308</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6326,41 +6398,77 @@
         <v>211</v>
       </c>
       <c r="B27" s="19" t="s">
-        <v>304</v>
+        <v>309</v>
       </c>
       <c r="C27" s="19" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="20"/>
-      <c r="B28" s="20"/>
-      <c r="C28" s="20"/>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="20"/>
-      <c r="B29" s="20"/>
-      <c r="C29" s="20"/>
+    <row r="28" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="19" t="s">
+        <v>231</v>
+      </c>
+      <c r="B28" s="19" t="s">
+        <v>310</v>
+      </c>
+      <c r="C28" s="19" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="19" t="s">
+        <v>231</v>
+      </c>
+      <c r="B29" s="19" t="s">
+        <v>312</v>
+      </c>
+      <c r="C29" s="19" t="s">
+        <v>313</v>
+      </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="20"/>
-      <c r="B30" s="20"/>
-      <c r="C30" s="20"/>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="20"/>
-      <c r="B31" s="20"/>
-      <c r="C31" s="20"/>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="20"/>
-      <c r="B32" s="20"/>
-      <c r="C32" s="20"/>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="20"/>
-      <c r="B33" s="20"/>
-      <c r="C33" s="20"/>
+      <c r="A30" s="19" t="s">
+        <v>231</v>
+      </c>
+      <c r="B30" s="19" t="s">
+        <v>314</v>
+      </c>
+      <c r="C30" s="19" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="19" t="s">
+        <v>231</v>
+      </c>
+      <c r="B31" s="19" t="s">
+        <v>315</v>
+      </c>
+      <c r="C31" s="19" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="19" t="s">
+        <v>231</v>
+      </c>
+      <c r="B32" s="19" t="s">
+        <v>317</v>
+      </c>
+      <c r="C32" s="19" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="19" t="s">
+        <v>231</v>
+      </c>
+      <c r="B33" s="19" t="s">
+        <v>319</v>
+      </c>
+      <c r="C33" s="19" t="s">
+        <v>320</v>
+      </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="20"/>
@@ -6406,6 +6514,36 @@
       <c r="A42" s="20"/>
       <c r="B42" s="20"/>
       <c r="C42" s="20"/>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="20"/>
+      <c r="B43" s="20"/>
+      <c r="C43" s="20"/>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="20"/>
+      <c r="B44" s="20"/>
+      <c r="C44" s="20"/>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="20"/>
+      <c r="B45" s="20"/>
+      <c r="C45" s="20"/>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="20"/>
+      <c r="B46" s="20"/>
+      <c r="C46" s="20"/>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="20"/>
+      <c r="B47" s="20"/>
+      <c r="C47" s="20"/>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="20"/>
+      <c r="B48" s="20"/>
+      <c r="C48" s="20"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -6437,19 +6575,19 @@
         <v>3</v>
       </c>
       <c r="B1" s="21" t="s">
-        <v>305</v>
+        <v>321</v>
       </c>
       <c r="C1" s="21" t="s">
-        <v>306</v>
+        <v>322</v>
       </c>
       <c r="D1" s="21" t="s">
         <v>10</v>
       </c>
       <c r="E1" s="21" t="s">
-        <v>307</v>
+        <v>323</v>
       </c>
       <c r="F1" s="21" t="s">
-        <v>308</v>
+        <v>324</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6497,7 +6635,7 @@
         <v>15</v>
       </c>
       <c r="B4" s="22" t="s">
-        <v>309</v>
+        <v>325</v>
       </c>
       <c r="C4" s="22" t="s">
         <v>61</v>
@@ -6511,7 +6649,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="22" t="s">
-        <v>235</v>
+        <v>241</v>
       </c>
       <c r="B5" s="22" t="s">
         <v>89</v>
@@ -6533,10 +6671,10 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="22" t="s">
-        <v>236</v>
+        <v>231</v>
       </c>
       <c r="B7" s="22" t="s">
-        <v>310</v>
+        <v>326</v>
       </c>
       <c r="C7" s="22" t="s">
         <v>49</v>
@@ -6544,7 +6682,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="22" t="s">
-        <v>237</v>
+        <v>242</v>
       </c>
       <c r="B8" s="22" t="s">
         <v>141</v>
@@ -6555,7 +6693,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="22" t="s">
-        <v>238</v>
+        <v>243</v>
       </c>
       <c r="C9" s="22" t="s">
         <v>30</v>
@@ -6563,7 +6701,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="22" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="C10" s="22" t="s">
         <v>126</v>

</xml_diff>